<commit_message>
Sync CPC projects under CPCs/, add Lead_Creation, and update case-shot automation.
Exclude local result zips/videos from git so the push stays within GitHub size limits.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/salesforce-case-shot/data/cases.xlsx
+++ b/salesforce-case-shot/data/cases.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dgosai\dhavalautomation-main\salesforce-case-shot\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABBE0BF5-7780-49D6-8359-93C15FFB713E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{143D6097-5934-4C96-9583-38DB9BC04BF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1815" yWindow="-14550" windowWidth="10200" windowHeight="11775" xr2:uid="{E95C6D45-A100-4653-92B2-89FF26A5E4F9}"/>
+    <workbookView xWindow="-20760" yWindow="4545" windowWidth="14400" windowHeight="7275" xr2:uid="{E95C6D45-A100-4653-92B2-89FF26A5E4F9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,48 +36,45 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Cases</t>
   </si>
   <si>
-    <t>00040658</t>
-  </si>
-  <si>
-    <t>00040660</t>
-  </si>
-  <si>
-    <t>00040661</t>
-  </si>
-  <si>
-    <t>00040662</t>
-  </si>
-  <si>
-    <t>00040663</t>
-  </si>
-  <si>
-    <t>00040664</t>
-  </si>
-  <si>
-    <t>00040659</t>
-  </si>
-  <si>
-    <t>00040665</t>
-  </si>
-  <si>
-    <t>00040666</t>
-  </si>
-  <si>
-    <t>00040667</t>
-  </si>
-  <si>
-    <t>00040668</t>
-  </si>
-  <si>
-    <t>00040669</t>
-  </si>
-  <si>
-    <t>00040677</t>
+    <t>00054828</t>
+  </si>
+  <si>
+    <t>00054829</t>
+  </si>
+  <si>
+    <t>00054830</t>
+  </si>
+  <si>
+    <t>00054831</t>
+  </si>
+  <si>
+    <t>00054833</t>
+  </si>
+  <si>
+    <t>00054835</t>
+  </si>
+  <si>
+    <t>00054836</t>
+  </si>
+  <si>
+    <t>00054837</t>
+  </si>
+  <si>
+    <t>00054838</t>
+  </si>
+  <si>
+    <t>00054839</t>
+  </si>
+  <si>
+    <t>00054841</t>
+  </si>
+  <si>
+    <t>00054844</t>
   </si>
 </sst>
 </file>
@@ -136,26 +133,25 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -490,7 +486,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88C08E2C-2410-414E-8B45-F07D7EB58B5F}">
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
@@ -499,38 +495,38 @@
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
-        <v>1</v>
+      <c r="A2" s="4" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
         <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
         <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A6" s="4" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
         <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A8" s="5" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.35">
@@ -549,7 +545,7 @@
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="3" t="s">
         <v>10</v>
       </c>
     </row>
@@ -558,14 +554,9 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A14" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:A11">
-    <sortCondition ref="A2:A11"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:A10">
+    <sortCondition ref="A2:A10"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>